<commit_message>
Scrub internal ST2 references from extenbook provenance cells
The 36 Extenbook .xlsx workbooks that ship a provenance note still
embedded internal predecessor-build references (`Inputs/ST2/...` cache
paths and bare `ST2`) inside their zipped sheet XML — the earlier
text-based scrub did not descend into the .xlsx binaries. Rewrote only
the affected XML members (surgical, no openpyxl round-trip: data,
styles, and structure preserved byte-for-byte) so the workbooks now use
the same public convention already applied to series_registry.json and
the data CSVs: `Inputs/ST2/` -> `data/raw/`, `ST2` -> `predecessor-build`.
No numeric values changed; all workbooks verified to open with intact
Data/Provenance/Research/Construction sheets.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/extenbooks/S401.xlsx
+++ b/extenbooks/S401.xlsx
@@ -938,7 +938,7 @@
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t>- Local files: `data/source/io_matrices/&lt;year&gt;_A_matrix.csv` (6 files copied from BEA Benchmark IO via ST2 IO_Matrices); printed-book digitization at `data/source/book_tables/ch04/Table4_1_AMatrix.csv`</t>
+          <t>- Local files: `data/source/io_matrices/&lt;year&gt;_A_matrix.csv` (6 files copied from BEA Benchmark IO via predecessor-build IO_Matrices); printed-book digitization at `data/source/book_tables/ch04/Table4_1_AMatrix.csv`</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
-          <t>- **Original research**: `Technical/research/S401_research.json`, researcher `agent`, 2026-05-06; ported from `ST2/research/T401_research.json` on 2026-05-14</t>
+          <t>- **Original research**: `Technical/research/S401_research.json`, researcher `agent`, 2026-05-06; ported from `predecessor-build/research/T401_research.json` on 2026-05-14</t>
         </is>
       </c>
     </row>

</xml_diff>